<commit_message>
Restore missing orders to Google Sheets and safeguard against full-sync overwriting
</commit_message>
<xml_diff>
--- a/납품대장.xlsx
+++ b/납품대장.xlsx
@@ -2459,7 +2459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L221"/>
+  <dimension ref="A1:L225"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.125" defaultRowHeight="16.5" customHeight="1"/>
   <cols>
     <col width="7.25" customWidth="1" style="21" min="1" max="1"/>
@@ -9614,29 +9614,29 @@
       </c>
     </row>
     <row r="220" ht="16.5" customHeight="1" s="141">
-      <c r="A220" t="n">
+      <c r="A220" s="131" t="n">
         <v>219</v>
       </c>
       <c r="B220" s="195" t="n">
         <v>46304</v>
       </c>
-      <c r="C220" t="inlineStr">
+      <c r="C220" s="131" t="inlineStr">
         <is>
           <t>화수브루어리</t>
         </is>
       </c>
-      <c r="D220" t="inlineStr">
-        <is>
-          <t>루꼴라</t>
-        </is>
-      </c>
-      <c r="E220" t="n">
+      <c r="D220" s="131" t="inlineStr">
+        <is>
+          <t>루꼴라</t>
+        </is>
+      </c>
+      <c r="E220" s="131" t="n">
         <v>17.7</v>
       </c>
-      <c r="F220" t="n">
+      <c r="F220" s="131" t="n">
         <v>300</v>
       </c>
-      <c r="G220" t="n">
+      <c r="G220" s="131" t="n">
         <v>5310</v>
       </c>
       <c r="H220" s="195" t="n">
@@ -9672,10 +9672,136 @@
         <v/>
       </c>
     </row>
-    <row r="222" ht="16.5" customHeight="1" s="141"/>
-    <row r="223" ht="16.5" customHeight="1" s="141"/>
-    <row r="224" ht="16.5" customHeight="1" s="141"/>
-    <row r="225" ht="16.5" customHeight="1" s="141"/>
+    <row r="222" ht="16.5" customHeight="1" s="141">
+      <c r="A222" t="n">
+        <v>221</v>
+      </c>
+      <c r="B222" s="195" t="n">
+        <v>46307</v>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>미즐 카페엠</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>루꼴라</t>
+        </is>
+      </c>
+      <c r="E222" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="F222" t="n">
+        <v>100</v>
+      </c>
+      <c r="G222" t="n">
+        <v>1770</v>
+      </c>
+      <c r="H222" s="195" t="n">
+        <v>46308</v>
+      </c>
+    </row>
+    <row r="223" ht="16.5" customHeight="1" s="141">
+      <c r="A223" t="n">
+        <v>222</v>
+      </c>
+      <c r="B223" s="195" t="n">
+        <v>46307</v>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>미즐 카페엠</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>엽채류</t>
+        </is>
+      </c>
+      <c r="E223" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="F223" t="n">
+        <v>100</v>
+      </c>
+      <c r="G223" t="n">
+        <v>1150</v>
+      </c>
+      <c r="H223" s="195" t="n">
+        <v>46308</v>
+      </c>
+      <c r="I223" t="inlineStr">
+        <is>
+          <t>프릴아이스</t>
+        </is>
+      </c>
+    </row>
+    <row r="224" ht="16.5" customHeight="1" s="141">
+      <c r="A224" t="n">
+        <v>223</v>
+      </c>
+      <c r="B224" s="195" t="n">
+        <v>46307</v>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>미즐 카페엠</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>엽채류</t>
+        </is>
+      </c>
+      <c r="E224" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="F224" t="n">
+        <v>100</v>
+      </c>
+      <c r="G224" t="n">
+        <v>1150</v>
+      </c>
+      <c r="H224" s="195" t="n">
+        <v>46308</v>
+      </c>
+      <c r="I224" t="inlineStr">
+        <is>
+          <t>이자트릭스</t>
+        </is>
+      </c>
+    </row>
+    <row r="225" ht="16.5" customHeight="1" s="141">
+      <c r="A225" t="n">
+        <v>224</v>
+      </c>
+      <c r="B225" s="195" t="n">
+        <v>46307</v>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>온터</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>딸기</t>
+        </is>
+      </c>
+      <c r="E225" t="n">
+        <v>50</v>
+      </c>
+      <c r="F225" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G225" t="n">
+        <v>50000</v>
+      </c>
+      <c r="H225" s="195" t="n">
+        <v>46308</v>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="A2:I991">
     <cfRule type="expression" priority="1" dxfId="0">

</xml_diff>

<commit_message>
Correct restored order: Birke Basil 1000g
</commit_message>
<xml_diff>
--- a/납품대장.xlsx
+++ b/납품대장.xlsx
@@ -9673,29 +9673,29 @@
       </c>
     </row>
     <row r="222" ht="16.5" customHeight="1" s="141">
-      <c r="A222" t="n">
+      <c r="A222" s="131" t="n">
         <v>221</v>
       </c>
       <c r="B222" s="195" t="n">
         <v>46307</v>
       </c>
-      <c r="C222" t="inlineStr">
+      <c r="C222" s="131" t="inlineStr">
         <is>
           <t>미즐 카페엠</t>
         </is>
       </c>
-      <c r="D222" t="inlineStr">
-        <is>
-          <t>루꼴라</t>
-        </is>
-      </c>
-      <c r="E222" t="n">
+      <c r="D222" s="131" t="inlineStr">
+        <is>
+          <t>루꼴라</t>
+        </is>
+      </c>
+      <c r="E222" s="131" t="n">
         <v>17.7</v>
       </c>
-      <c r="F222" t="n">
+      <c r="F222" s="131" t="n">
         <v>100</v>
       </c>
-      <c r="G222" t="n">
+      <c r="G222" s="131" t="n">
         <v>1770</v>
       </c>
       <c r="H222" s="195" t="n">
@@ -9703,100 +9703,100 @@
       </c>
     </row>
     <row r="223" ht="16.5" customHeight="1" s="141">
-      <c r="A223" t="n">
+      <c r="A223" s="131" t="n">
         <v>222</v>
       </c>
       <c r="B223" s="195" t="n">
         <v>46307</v>
       </c>
-      <c r="C223" t="inlineStr">
+      <c r="C223" s="131" t="inlineStr">
         <is>
           <t>미즐 카페엠</t>
         </is>
       </c>
-      <c r="D223" t="inlineStr">
+      <c r="D223" s="131" t="inlineStr">
         <is>
           <t>엽채류</t>
         </is>
       </c>
-      <c r="E223" t="n">
+      <c r="E223" s="131" t="n">
         <v>11.5</v>
       </c>
-      <c r="F223" t="n">
+      <c r="F223" s="131" t="n">
         <v>100</v>
       </c>
-      <c r="G223" t="n">
+      <c r="G223" s="131" t="n">
         <v>1150</v>
       </c>
       <c r="H223" s="195" t="n">
         <v>46308</v>
       </c>
-      <c r="I223" t="inlineStr">
+      <c r="I223" s="131" t="inlineStr">
         <is>
           <t>프릴아이스</t>
         </is>
       </c>
     </row>
     <row r="224" ht="16.5" customHeight="1" s="141">
-      <c r="A224" t="n">
+      <c r="A224" s="131" t="n">
         <v>223</v>
       </c>
       <c r="B224" s="195" t="n">
         <v>46307</v>
       </c>
-      <c r="C224" t="inlineStr">
+      <c r="C224" s="131" t="inlineStr">
         <is>
           <t>미즐 카페엠</t>
         </is>
       </c>
-      <c r="D224" t="inlineStr">
+      <c r="D224" s="131" t="inlineStr">
         <is>
           <t>엽채류</t>
         </is>
       </c>
-      <c r="E224" t="n">
+      <c r="E224" s="131" t="n">
         <v>11.5</v>
       </c>
-      <c r="F224" t="n">
+      <c r="F224" s="131" t="n">
         <v>100</v>
       </c>
-      <c r="G224" t="n">
+      <c r="G224" s="131" t="n">
         <v>1150</v>
       </c>
       <c r="H224" s="195" t="n">
         <v>46308</v>
       </c>
-      <c r="I224" t="inlineStr">
+      <c r="I224" s="131" t="inlineStr">
         <is>
           <t>이자트릭스</t>
         </is>
       </c>
     </row>
     <row r="225" ht="16.5" customHeight="1" s="141">
-      <c r="A225" t="n">
+      <c r="A225" s="131" t="n">
         <v>224</v>
       </c>
       <c r="B225" s="195" t="n">
         <v>46307</v>
       </c>
-      <c r="C225" t="inlineStr">
-        <is>
-          <t>온터</t>
-        </is>
-      </c>
-      <c r="D225" t="inlineStr">
-        <is>
-          <t>딸기</t>
-        </is>
-      </c>
-      <c r="E225" t="n">
-        <v>50</v>
-      </c>
-      <c r="F225" t="n">
+      <c r="C225" s="131" t="inlineStr">
+        <is>
+          <t>비르케</t>
+        </is>
+      </c>
+      <c r="D225" s="131" t="inlineStr">
+        <is>
+          <t>바질</t>
+        </is>
+      </c>
+      <c r="E225" s="131" t="n">
+        <v>35</v>
+      </c>
+      <c r="F225" s="131" t="n">
         <v>1000</v>
       </c>
-      <c r="G225" t="n">
-        <v>50000</v>
+      <c r="G225" s="131" t="n">
+        <v>35000</v>
       </c>
       <c r="H225" s="195" t="n">
         <v>46308</v>

</xml_diff>

<commit_message>
Fix order edit sync to Google Sheets and simplify receipt cut line to single line
</commit_message>
<xml_diff>
--- a/납품대장.xlsx
+++ b/납품대장.xlsx
@@ -9773,29 +9773,29 @@
       </c>
     </row>
     <row r="225" ht="16.5" customHeight="1" s="141">
-      <c r="A225" s="131" t="n">
+      <c r="A225" t="n">
         <v>224</v>
       </c>
       <c r="B225" s="195" t="n">
         <v>46307</v>
       </c>
-      <c r="C225" s="131" t="inlineStr">
+      <c r="C225" t="inlineStr">
         <is>
           <t>비르케</t>
         </is>
       </c>
-      <c r="D225" s="131" t="inlineStr">
+      <c r="D225" t="inlineStr">
         <is>
           <t>바질</t>
         </is>
       </c>
-      <c r="E225" s="131" t="n">
+      <c r="E225" t="n">
         <v>35</v>
       </c>
-      <c r="F225" s="131" t="n">
+      <c r="F225" t="n">
         <v>1000</v>
       </c>
-      <c r="G225" s="131" t="n">
+      <c r="G225" t="n">
         <v>35000</v>
       </c>
       <c r="H225" s="195" t="n">

</xml_diff>